<commit_message>
Add September 2026 data and report title to auto transport report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUGocJva82HrAiQV6F1p2k
</commit_message>
<xml_diff>
--- a/out/Отчет_заявки_и_обеспечение_2026.xlsx
+++ b/out/Отчет_заявки_и_обеспечение_2026.xlsx
@@ -19,13 +19,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -76,24 +81,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -472,716 +480,790 @@
     <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Филиал Кока-кола Алматы Боттлерс СП ТОО г. Астана — январь–август 2026 г.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+          <t>Отчет по автоперевозкам: заявки и обеспечение за январь–сентябрь 2026 г.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Филиал Кока-кола Алматы Боттлерс СП ТОО г. Астана — январь–сентябрь 2026 г.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Количество заявок</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Обеспечение</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Отгрузка Zhebe Logistics</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>% выполнения по заявке</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
+    <row r="5">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Январь</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C5" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.6486486486486487</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
+    <row r="6">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Февраль</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C6" s="4" t="n">
         <v>324</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D6" s="4" t="n">
         <v>178</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E6" s="4" t="n">
         <v>178</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.5493827160493827</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
+    <row r="7">
+      <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Март</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C7" s="4" t="n">
         <v>124</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D7" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E7" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.6370967741935484</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
+    <row r="8">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Апрель</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C8" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D8" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E8" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.6333333333333333</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
+    <row r="9">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Май</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C9" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
+    <row r="10">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Июнь</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C10" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D10" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F10" s="5" t="n">
         <v>0.3333333333333333</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
+    <row r="11">
+      <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Июль</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C11" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D11" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E11" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
+    <row r="12">
+      <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Август</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C12" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E12" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F12" s="5" t="n">
         <v>0.08888888888888889</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Сентябрь</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.1818181818181818</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
-        <v>713</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>373</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>373</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>0.5231416549789621</v>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Кока-кола Алматы Боттлерс СП ТОО АЛМАТЫ, Бурундай — январь–август 2026 г.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="C14" s="6" t="n">
+        <v>724</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>375</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>375</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0.5179558011049724</v>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Кока-кола Алматы Боттлерс СП ТОО АЛМАТЫ, Бурундай — январь–сентябрь 2026 г.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Количество заявок</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Обеспечение</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Отгрузка Zhebe Logistics</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>% выполнения по заявке</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
+    <row r="19">
+      <c r="A19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Январь</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C19" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D19" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E19" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F19" s="5" t="n">
         <v>0.2608695652173913</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
+    <row r="20">
+      <c r="A20" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Февраль</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C20" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D20" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E20" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F20" s="5" t="n">
         <v>0.36</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="n">
+    <row r="21">
+      <c r="A21" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Март</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C21" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D21" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E21" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="F21" s="5" t="n">
         <v>0.5212765957446809</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="n">
+    <row r="22">
+      <c r="A22" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Апрель</t>
         </is>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C22" s="4" t="n">
         <v>111</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D22" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E22" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="F22" s="5" t="n">
         <v>0.6756756756756757</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="n">
+    <row r="23">
+      <c r="A23" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Май</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C23" s="4" t="n">
         <v>252</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D23" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E23" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="F23" s="5" t="n">
         <v>0.5079365079365079</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
+    <row r="24">
+      <c r="A24" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Июнь</t>
         </is>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C24" s="4" t="n">
         <v>268</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D24" s="4" t="n">
         <v>91</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E24" s="4" t="n">
         <v>91</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F24" s="5" t="n">
         <v>0.3395522388059701</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
+    <row r="25">
+      <c r="A25" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Июль</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D25" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E25" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="F25" s="5" t="n">
         <v>0.5416666666666666</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
+    <row r="26">
+      <c r="A26" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Август</t>
         </is>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C26" s="4" t="n">
         <v>188</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D26" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E26" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="F26" s="5" t="n">
         <v>0.1170212765957447</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Сентябрь</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0.4953271028037383</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr"/>
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C24" s="5" t="n">
-        <v>1010</v>
-      </c>
-      <c r="D24" s="5" t="n">
-        <v>402</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>402</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>0.398019801980198</v>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Филиал Кока-кола Алматы Боттлерс СП ТОО г. Шымкент — январь–август 2026 г.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="C28" s="6" t="n">
+        <v>1117</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>455</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>455</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>0.4073410922112802</v>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Филиал Кока-кола Алматы Боттлерс СП ТОО г. Шымкент — январь–сентябрь 2026 г.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Количество заявок</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Обеспечение</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Отгрузка Zhebe Logistics</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>% выполнения по заявке</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="n">
+    <row r="33">
+      <c r="A33" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Январь</t>
         </is>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C33" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="E33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="F33" s="5" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="n">
+    <row r="34">
+      <c r="A34" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Февраль</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C34" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D34" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E34" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="F30" s="4" t="n">
+      <c r="F34" s="5" t="n">
         <v>0.4328358208955224</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="n">
+    <row r="35">
+      <c r="A35" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Март</t>
         </is>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C35" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D35" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E31" s="3" t="n">
+      <c r="E35" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="F35" s="5" t="n">
         <v>0.631578947368421</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="n">
+    <row r="36">
+      <c r="A36" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Апрель</t>
         </is>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C36" s="4" t="n">
         <v>133</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D36" s="4" t="n">
         <v>83</v>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="E36" s="4" t="n">
         <v>83</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="F36" s="5" t="n">
         <v>0.6240601503759399</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="n">
+    <row r="37">
+      <c r="A37" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Май</t>
         </is>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C37" s="4" t="n">
         <v>397</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D37" s="4" t="n">
         <v>176</v>
       </c>
-      <c r="E33" s="3" t="n">
+      <c r="E37" s="4" t="n">
         <v>176</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="F37" s="5" t="n">
         <v>0.4433249370277078</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="n">
+    <row r="38">
+      <c r="A38" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Июнь</t>
         </is>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C38" s="4" t="n">
         <v>628</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D38" s="4" t="n">
         <v>328</v>
       </c>
-      <c r="E34" s="3" t="n">
+      <c r="E38" s="4" t="n">
         <v>328</v>
       </c>
-      <c r="F34" s="4" t="n">
+      <c r="F38" s="5" t="n">
         <v>0.5222929936305732</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="n">
+    <row r="39">
+      <c r="A39" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Июль</t>
         </is>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C39" s="4" t="n">
         <v>635</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D39" s="4" t="n">
         <v>343</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E39" s="4" t="n">
         <v>343</v>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="F39" s="5" t="n">
         <v>0.5401574803149606</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="n">
+    <row r="40">
+      <c r="A40" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Август</t>
         </is>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C40" s="4" t="n">
         <v>162</v>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D40" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="E36" s="3" t="n">
+      <c r="E40" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="F36" s="4" t="n">
+      <c r="F40" s="5" t="n">
         <v>0.4012345679012346</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr"/>
-      <c r="B37" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Сентябрь</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0.1904761904761905</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr"/>
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C37" s="5" t="n">
-        <v>2044</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>1036</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>1036</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>0.5068493150684932</v>
+      <c r="C42" s="6" t="n">
+        <v>2065</v>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>1040</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>0.5036319612590799</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A14:F14"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add monthly averages and combined all-branch report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUGocJva82HrAiQV6F1p2k
</commit_message>
<xml_diff>
--- a/out/Отчет_заявки_и_обеспечение_2026.xlsx
+++ b/out/Отчет_заявки_и_обеспечение_2026.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -45,7 +46,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -81,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -95,13 +101,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -469,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -535,16 +556,16 @@
           <t>Январь</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <v>0.6486486486486487</v>
       </c>
     </row>
@@ -557,16 +578,16 @@
           <t>Февраль</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>324</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>178</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>178</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
         <v>0.5493827160493827</v>
       </c>
     </row>
@@ -579,16 +600,16 @@
           <t>Март</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>124</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>79</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>79</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="6" t="n">
         <v>0.6370967741935484</v>
       </c>
     </row>
@@ -601,16 +622,16 @@
           <t>Апрель</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="6" t="n">
         <v>0.6333333333333333</v>
       </c>
     </row>
@@ -623,16 +644,16 @@
           <t>Май</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="6" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -645,16 +666,16 @@
           <t>Июнь</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="5" t="n">
         <v>69</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
     </row>
@@ -667,16 +688,16 @@
           <t>Июль</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="6" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -689,16 +710,16 @@
           <t>Август</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="6" t="n">
         <v>0.08888888888888889</v>
       </c>
     </row>
@@ -711,559 +732,622 @@
           <t>Сентябрь</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F13" s="6" t="n">
         <v>0.1818181818181818</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr"/>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>СРЕДНЕЕ
+(в месяц)</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0.4525002084739241</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C15" s="11" t="n">
         <v>724</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D15" s="11" t="n">
         <v>375</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E15" s="11" t="n">
         <v>375</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F15" s="12" t="n">
         <v>0.5179558011049724</v>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Кока-кола Алматы Боттлерс СП ТОО АЛМАТЫ, Бурундай — январь–сентябрь 2026 г.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Количество заявок</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Обеспечение</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Отгрузка Zhebe Logistics</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>% выполнения по заявке</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Январь</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0.2608695652173913</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Февраль</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>0.36</v>
+          <t>Январь</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>0.2608695652173913</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Март</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>94</v>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>0.5212765957446809</v>
+          <t>Февраль</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0.36</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Апрель</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>111</v>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>0.6756756756756757</v>
+          <t>Март</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>0.5212765957446809</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Май</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="n">
-        <v>252</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>128</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>128</v>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>0.5079365079365079</v>
+          <t>Апрель</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>111</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>0.6756756756756757</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Июнь</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>268</v>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>91</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>91</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>0.3395522388059701</v>
+          <t>Май</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>252</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>128</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>128</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>0.5079365079365079</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Июль</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>0.5416666666666666</v>
+          <t>Июнь</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>268</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0.3395522388059701</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Август</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>188</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F26" s="5" t="n">
-        <v>0.1170212765957447</v>
+          <t>Июль</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0.5416666666666666</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Август</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0.1170212765957447</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Сентябрь</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C28" s="5" t="n">
         <v>107</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D28" s="5" t="n">
         <v>53</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E28" s="5" t="n">
         <v>53</v>
       </c>
-      <c r="F27" s="5" t="n">
+      <c r="F28" s="6" t="n">
         <v>0.4953271028037383</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr"/>
-      <c r="B28" s="6" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>СРЕДНЕЕ
+(в месяц)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>124.1</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>0.4243695143829306</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr"/>
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C30" s="11" t="n">
         <v>1117</v>
       </c>
-      <c r="D28" s="6" t="n">
+      <c r="D30" s="11" t="n">
         <v>455</v>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="E30" s="11" t="n">
         <v>455</v>
       </c>
-      <c r="F28" s="7" t="n">
+      <c r="F30" s="12" t="n">
         <v>0.4073410922112802</v>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Филиал Кока-кола Алматы Боттлерс СП ТОО г. Шымкент — январь–сентябрь 2026 г.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Количество заявок</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Обеспечение</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>Отгрузка Zhebe Logistics</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>% выполнения по заявке</t>
         </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Январь</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Февраль</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>67</v>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>0.4328358208955224</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Январь</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Март</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>0.631578947368421</v>
+      <c r="D35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Апрель</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="n">
-        <v>133</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>0.6240601503759399</v>
+          <t>Февраль</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>0.4328358208955224</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Май</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>397</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>176</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>176</v>
-      </c>
-      <c r="F37" s="5" t="n">
-        <v>0.4433249370277078</v>
+          <t>Март</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>0.631578947368421</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Июнь</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>628</v>
-      </c>
-      <c r="D38" s="4" t="n">
-        <v>328</v>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>328</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>0.5222929936305732</v>
+          <t>Апрель</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>133</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>0.6240601503759399</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Июль</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="n">
-        <v>635</v>
-      </c>
-      <c r="D39" s="4" t="n">
-        <v>343</v>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>343</v>
-      </c>
-      <c r="F39" s="5" t="n">
-        <v>0.5401574803149606</v>
+          <t>Май</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>397</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>176</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>176</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>0.4433249370277078</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Август</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>162</v>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="F40" s="5" t="n">
-        <v>0.4012345679012346</v>
+          <t>Июнь</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>628</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>328</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>328</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>0.5222929936305732</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Июль</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>635</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>343</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>343</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0.5401574803149606</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Август</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>162</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>0.4012345679012346</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Сентябрь</t>
         </is>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C43" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="D43" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E43" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F41" s="5" t="n">
+      <c r="F43" s="6" t="n">
         <v>0.1904761904761905</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr"/>
-      <c r="B42" s="6" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr"/>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>СРЕДНЕЕ
+(в месяц)</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n">
+        <v>229.4</v>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>0.4206623431100611</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr"/>
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C42" s="6" t="n">
+      <c r="C45" s="11" t="n">
         <v>2065</v>
       </c>
-      <c r="D42" s="6" t="n">
+      <c r="D45" s="11" t="n">
         <v>1040</v>
       </c>
-      <c r="E42" s="6" t="n">
+      <c r="E45" s="11" t="n">
         <v>1040</v>
       </c>
-      <c r="F42" s="7" t="n">
+      <c r="F45" s="12" t="n">
         <v>0.5036319612590799</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A33:F33"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>